<commit_message>
Add 12-month price targets, bull/bear scenarios and relative ratings
models/target.py: fair value = DCF + comps blend (comps only where the DCF is
not meaningful), rolled forward a year at the cost of equity and rounded.
Bull/bear shift DCF growth and mature margin and move the comps multiple by
one residual s.d. of the peer regression (0.56 in log terms). Ratings are
Overweight/Neutral/Underweight relative to the coverage median; targets
beyond +/-75% are flagged as model outliers, not capped. All in config.yaml.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/comps_CY2025.xlsx
+++ b/outputs/comps_CY2025.xlsx
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Calendarized to CY2025 · Market data as of 2026-10-18 · $ in millions except per-share · NM = not meaningful, n/a = missing input</t>
+          <t>Calendarized to CY2025 · Market data as of 2026-11-01 · $ in millions except per-share · NM = not meaningful, n/a = missing input</t>
         </is>
       </c>
     </row>
@@ -571,22 +571,22 @@
         </is>
       </c>
       <c r="D5" s="5" t="n">
-        <v>245.2</v>
+        <v>250.23</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>95431.83564799999</v>
+        <v>97389.510656</v>
       </c>
       <c r="F5" s="6" t="n">
-        <v>95046.83564799999</v>
+        <v>97004.510656</v>
       </c>
       <c r="G5" s="7" t="n">
-        <v>3.998773008877109</v>
+        <v>4.081135540241491</v>
       </c>
       <c r="H5" s="7" t="n">
-        <v>9.979718148677026</v>
+        <v>10.18526991348173</v>
       </c>
       <c r="I5" s="7" t="n">
-        <v>9.686544422249289</v>
+        <v>9.885252807145758</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
@@ -611,22 +611,22 @@
         </is>
       </c>
       <c r="D6" s="5" t="n">
-        <v>240.7</v>
+        <v>229.17</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>198096.093184</v>
+        <v>188606.906368</v>
       </c>
       <c r="F6" s="6" t="n">
-        <v>202970.093184</v>
+        <v>193480.906368</v>
       </c>
       <c r="G6" s="7" t="n">
-        <v>4.923769620571291</v>
+        <v>4.693575265158591</v>
       </c>
       <c r="H6" s="7" t="n">
-        <v>21.54557541361924</v>
+        <v>20.53828420657078</v>
       </c>
       <c r="I6" s="7" t="n">
-        <v>13.91319659952241</v>
+        <v>13.24672751566231</v>
       </c>
       <c r="J6" t="inlineStr"/>
     </row>
@@ -647,16 +647,16 @@
         </is>
       </c>
       <c r="D7" s="5" t="n">
-        <v>227.39</v>
+        <v>250.43</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>232832.548864</v>
+        <v>256424.001536</v>
       </c>
       <c r="F7" s="6" t="n">
-        <v>228347.894864</v>
+        <v>251939.347536</v>
       </c>
       <c r="G7" s="7" t="n">
-        <v>48.16985200032507</v>
+        <v>53.14645484730876</v>
       </c>
       <c r="H7" s="8" t="inlineStr">
         <is>
@@ -691,16 +691,16 @@
         </is>
       </c>
       <c r="D8" s="5" t="n">
-        <v>247.11</v>
+        <v>235.27</v>
       </c>
       <c r="E8" s="6" t="n">
-        <v>88731.025408</v>
+        <v>84479.58220800001</v>
       </c>
       <c r="F8" s="6" t="n">
-        <v>85239.638408</v>
+        <v>80988.195208</v>
       </c>
       <c r="G8" s="7" t="n">
-        <v>24.87181460790544</v>
+        <v>23.63129893865413</v>
       </c>
       <c r="H8" s="8" t="inlineStr">
         <is>
@@ -708,7 +708,7 @@
         </is>
       </c>
       <c r="I8" s="7" t="n">
-        <v>97.00380052846945</v>
+        <v>92.35597699397738</v>
       </c>
       <c r="J8" t="inlineStr"/>
     </row>
@@ -729,22 +729,22 @@
         </is>
       </c>
       <c r="D9" s="5" t="n">
-        <v>74.65000000000001</v>
+        <v>82.17</v>
       </c>
       <c r="E9" s="6" t="n">
-        <v>13952.268288</v>
+        <v>15357.773824</v>
       </c>
       <c r="F9" s="6" t="n">
-        <v>13349.826288</v>
+        <v>14755.331824</v>
       </c>
       <c r="G9" s="7" t="n">
-        <v>4.172772737446687</v>
+        <v>4.612093448924637</v>
       </c>
       <c r="H9" s="7" t="n">
-        <v>32.90165920502642</v>
+        <v>36.36563417808039</v>
       </c>
       <c r="I9" s="7" t="n">
-        <v>13.32545445671945</v>
+        <v>14.66781683264533</v>
       </c>
       <c r="J9" t="inlineStr">
         <is>
@@ -769,22 +769,22 @@
         </is>
       </c>
       <c r="D10" s="5" t="n">
-        <v>230.94</v>
+        <v>234.87</v>
       </c>
       <c r="E10" s="6" t="n">
-        <v>11516.100608</v>
+        <v>11712.073728</v>
       </c>
       <c r="F10" s="6" t="n">
-        <v>9812.306608000001</v>
+        <v>10008.279728</v>
       </c>
       <c r="G10" s="7" t="n">
-        <v>3.133654760726173</v>
+        <v>3.196240666874038</v>
       </c>
       <c r="H10" s="7" t="n">
-        <v>68.29563183317789</v>
+        <v>69.65964425017748</v>
       </c>
       <c r="I10" s="7" t="n">
-        <v>19.96107071939653</v>
+        <v>20.3007545620944</v>
       </c>
       <c r="J10" t="inlineStr">
         <is>
@@ -809,16 +809,16 @@
         </is>
       </c>
       <c r="D11" s="5" t="n">
-        <v>337.57</v>
+        <v>352.96</v>
       </c>
       <c r="E11" s="6" t="n">
-        <v>27193.40544</v>
+        <v>28433.166336</v>
       </c>
       <c r="F11" s="6" t="n">
-        <v>24806.16444</v>
+        <v>26045.925336</v>
       </c>
       <c r="G11" s="7" t="n">
-        <v>10.22646096341891</v>
+        <v>10.73755837380588</v>
       </c>
       <c r="H11" s="8" t="inlineStr">
         <is>
@@ -826,7 +826,7 @@
         </is>
       </c>
       <c r="I11" s="7" t="n">
-        <v>58.03623578598857</v>
+        <v>60.68213667682251</v>
       </c>
       <c r="J11" t="inlineStr">
         <is>
@@ -851,22 +851,22 @@
         </is>
       </c>
       <c r="D12" s="5" t="n">
-        <v>141.97</v>
+        <v>105.12</v>
       </c>
       <c r="E12" s="6" t="n">
-        <v>146777.391104</v>
+        <v>109105.840128</v>
       </c>
       <c r="F12" s="6" t="n">
-        <v>141984.391104</v>
+        <v>104312.840128</v>
       </c>
       <c r="G12" s="7" t="n">
-        <v>10.69320613827384</v>
+        <v>7.856065682181051</v>
       </c>
       <c r="H12" s="7" t="n">
-        <v>55.4193564028103</v>
+        <v>40.71539427322404</v>
       </c>
       <c r="I12" s="7" t="n">
-        <v>32.07547882517483</v>
+        <v>23.84305946853147</v>
       </c>
       <c r="J12" t="inlineStr">
         <is>
@@ -891,16 +891,16 @@
         </is>
       </c>
       <c r="D13" s="5" t="n">
-        <v>187.26</v>
+        <v>208.24</v>
       </c>
       <c r="E13" s="6" t="n">
-        <v>32736.966656</v>
+        <v>36404.711424</v>
       </c>
       <c r="F13" s="6" t="n">
-        <v>32228.966656</v>
+        <v>35896.711424</v>
       </c>
       <c r="G13" s="7" t="n">
-        <v>11.13936460934935</v>
+        <v>12.40705484282381</v>
       </c>
       <c r="H13" s="8" t="inlineStr">
         <is>
@@ -908,7 +908,7 @@
         </is>
       </c>
       <c r="I13" s="7" t="n">
-        <v>38.42742833532231</v>
+        <v>42.73271418252959</v>
       </c>
       <c r="J13" t="inlineStr"/>
     </row>
@@ -929,22 +929,22 @@
         </is>
       </c>
       <c r="D14" s="5" t="n">
-        <v>251.64</v>
+        <v>264.2</v>
       </c>
       <c r="E14" s="6" t="n">
-        <v>11341.821952</v>
+        <v>11907.922944</v>
       </c>
       <c r="F14" s="6" t="n">
-        <v>10971.821952</v>
+        <v>11537.922944</v>
       </c>
       <c r="G14" s="7" t="n">
-        <v>5.347673613101331</v>
+        <v>5.623591628405713</v>
       </c>
       <c r="H14" s="7" t="n">
-        <v>14.75698984801614</v>
+        <v>15.51838997175521</v>
       </c>
       <c r="I14" s="7" t="n">
-        <v>27.79858321568627</v>
+        <v>29.18608564705882</v>
       </c>
       <c r="J14" t="inlineStr">
         <is>
@@ -969,22 +969,22 @@
         </is>
       </c>
       <c r="D15" s="5" t="n">
-        <v>166.32</v>
+        <v>170.91</v>
       </c>
       <c r="E15" s="6" t="n">
-        <v>8824.434687999999</v>
+        <v>8917.103616</v>
       </c>
       <c r="F15" s="6" t="n">
-        <v>8633.767688</v>
+        <v>8726.436616000001</v>
       </c>
       <c r="G15" s="7" t="n">
-        <v>5.129153217228216</v>
+        <v>5.184206022372479</v>
       </c>
       <c r="H15" s="7" t="n">
-        <v>19.15528911864219</v>
+        <v>19.36088882578069</v>
       </c>
       <c r="I15" s="7" t="n">
-        <v>22.90427912566235</v>
+        <v>23.14480614730536</v>
       </c>
       <c r="J15" t="inlineStr"/>
     </row>
@@ -1005,16 +1005,16 @@
         </is>
       </c>
       <c r="D16" s="5" t="n">
-        <v>306.84</v>
+        <v>306.08</v>
       </c>
       <c r="E16" s="6" t="n">
-        <v>108253.151232</v>
+        <v>107985.01888</v>
       </c>
       <c r="F16" s="6" t="n">
-        <v>106503.292232</v>
+        <v>106235.15988</v>
       </c>
       <c r="G16" s="7" t="n">
-        <v>23.17396364875435</v>
+        <v>23.11562095109607</v>
       </c>
       <c r="H16" s="8" t="inlineStr">
         <is>
@@ -1022,7 +1022,7 @@
         </is>
       </c>
       <c r="I16" s="7" t="n">
-        <v>98.35602685200371</v>
+        <v>98.11240869850826</v>
       </c>
       <c r="J16" t="inlineStr"/>
     </row>
@@ -1043,16 +1043,16 @@
         </is>
       </c>
       <c r="D17" s="5" t="n">
-        <v>207.82</v>
+        <v>191.72</v>
       </c>
       <c r="E17" s="6" t="n">
-        <v>52607.311872</v>
+        <v>48531.775488</v>
       </c>
       <c r="F17" s="6" t="n">
-        <v>52357.359872</v>
+        <v>48281.823488</v>
       </c>
       <c r="G17" s="7" t="n">
-        <v>8.883454913853628</v>
+        <v>8.191960082839509</v>
       </c>
       <c r="H17" s="8" t="inlineStr">
         <is>
@@ -1060,7 +1060,7 @@
         </is>
       </c>
       <c r="I17" s="7" t="n">
-        <v>38.47507174457273</v>
+        <v>35.49437287986841</v>
       </c>
       <c r="J17" t="inlineStr"/>
     </row>
@@ -1081,24 +1081,22 @@
         </is>
       </c>
       <c r="D18" s="5" t="n">
-        <v>244.37</v>
+        <v>205.03</v>
       </c>
       <c r="E18" s="6" t="n">
-        <v>37529.174016</v>
+        <v>31487.526912</v>
       </c>
       <c r="F18" s="6" t="n">
-        <v>36051.119016</v>
+        <v>30009.471912</v>
       </c>
       <c r="G18" s="7" t="n">
-        <v>7.114575450838921</v>
-      </c>
-      <c r="H18" s="8" t="inlineStr">
-        <is>
-          <t>NM</t>
-        </is>
+        <v>5.922275313090807</v>
+      </c>
+      <c r="H18" s="7" t="n">
+        <v>84.95346560753696</v>
       </c>
       <c r="I18" s="7" t="n">
-        <v>39.6954751831712</v>
+        <v>33.30508533392848</v>
       </c>
       <c r="J18" t="inlineStr"/>
     </row>
@@ -1119,22 +1117,22 @@
         </is>
       </c>
       <c r="D19" s="5" t="n">
-        <v>310.36</v>
+        <v>312.96</v>
       </c>
       <c r="E19" s="6" t="n">
-        <v>50250.027008</v>
+        <v>50670.993408</v>
       </c>
       <c r="F19" s="6" t="n">
-        <v>43689.213008</v>
+        <v>44110.179408</v>
       </c>
       <c r="G19" s="7" t="n">
-        <v>13.83480677407914</v>
+        <v>13.96811173430613</v>
       </c>
       <c r="H19" s="7" t="n">
-        <v>46.69077209179549</v>
+        <v>47.14065994482467</v>
       </c>
       <c r="I19" s="7" t="n">
-        <v>36.95632549741165</v>
+        <v>37.26592475990353</v>
       </c>
       <c r="J19" t="inlineStr">
         <is>
@@ -1159,22 +1157,22 @@
         </is>
       </c>
       <c r="D20" s="5" t="n">
-        <v>190.81</v>
+        <v>197.82</v>
       </c>
       <c r="E20" s="6" t="n">
-        <v>45985.210368</v>
+        <v>47674.621952</v>
       </c>
       <c r="F20" s="6" t="n">
-        <v>43529.210368</v>
+        <v>45218.621952</v>
       </c>
       <c r="G20" s="7" t="n">
-        <v>4.601477513839215</v>
+        <v>4.780065394245846</v>
       </c>
       <c r="H20" s="7" t="n">
-        <v>41.82484781936104</v>
+        <v>43.44811141196253</v>
       </c>
       <c r="I20" s="7" t="n">
-        <v>16.85520402015944</v>
+        <v>17.47443304389261</v>
       </c>
       <c r="J20" t="inlineStr">
         <is>
@@ -1199,22 +1197,22 @@
         </is>
       </c>
       <c r="D21" s="5" t="n">
-        <v>94.19</v>
+        <v>95.5</v>
       </c>
       <c r="E21" s="6" t="n">
-        <v>27483.109376</v>
+        <v>27865.344</v>
       </c>
       <c r="F21" s="6" t="n">
-        <v>19666.201376</v>
+        <v>20048.436</v>
       </c>
       <c r="G21" s="7" t="n">
-        <v>4.053362204581053</v>
+        <v>4.13214383345701</v>
       </c>
       <c r="H21" s="7" t="n">
-        <v>15.99199842515747</v>
+        <v>16.30282080453717</v>
       </c>
       <c r="I21" s="7" t="n">
-        <v>14.35542558381419</v>
+        <v>14.55508060193164</v>
       </c>
       <c r="J21" t="inlineStr">
         <is>
@@ -1239,16 +1237,16 @@
         </is>
       </c>
       <c r="D22" s="5" t="n">
-        <v>207.38</v>
+        <v>237.83</v>
       </c>
       <c r="E22" s="6" t="n">
-        <v>33814.284288</v>
+        <v>38779.301888</v>
       </c>
       <c r="F22" s="6" t="n">
-        <v>34582.285288</v>
+        <v>39547.302888</v>
       </c>
       <c r="G22" s="7" t="n">
-        <v>11.6982158822047</v>
+        <v>13.37774189559688</v>
       </c>
       <c r="H22" s="8" t="inlineStr">
         <is>
@@ -1256,7 +1254,7 @@
         </is>
       </c>
       <c r="I22" s="7" t="n">
-        <v>45.17321792636981</v>
+        <v>51.80609000323515</v>
       </c>
       <c r="J22" t="inlineStr"/>
     </row>
@@ -1272,13 +1270,13 @@
       <c r="E24" s="10" t="n"/>
       <c r="F24" s="10" t="n"/>
       <c r="G24" s="11" t="n">
-        <v>48.16985200032507</v>
+        <v>53.14645484730876</v>
       </c>
       <c r="H24" s="11" t="n">
-        <v>68.29563183317789</v>
+        <v>84.95346560753696</v>
       </c>
       <c r="I24" s="11" t="n">
-        <v>98.35602685200371</v>
+        <v>98.11240869850826</v>
       </c>
       <c r="J24" s="10" t="n"/>
     </row>
@@ -1294,13 +1292,13 @@
       <c r="E25" s="10" t="n"/>
       <c r="F25" s="10" t="n"/>
       <c r="G25" s="11" t="n">
-        <v>11.55850306399086</v>
+        <v>13.13507013240362</v>
       </c>
       <c r="H25" s="11" t="n">
-        <v>45.47429102368687</v>
+        <v>45.2943856783936</v>
       </c>
       <c r="I25" s="11" t="n">
-        <v>39.6954751831712</v>
+        <v>42.73271418252959</v>
       </c>
       <c r="J25" s="10" t="n"/>
     </row>
@@ -1316,13 +1314,13 @@
       <c r="E26" s="10" t="n"/>
       <c r="F26" s="10" t="n"/>
       <c r="G26" s="11" t="n">
-        <v>11.39813064807636</v>
+        <v>11.59206635896571</v>
       </c>
       <c r="H26" s="11" t="n">
-        <v>32.65618383062832</v>
+        <v>36.74441485344834</v>
       </c>
       <c r="I26" s="11" t="n">
-        <v>36.64698934245261</v>
+        <v>36.35639565617888</v>
       </c>
       <c r="J26" s="10" t="n"/>
     </row>
@@ -1338,13 +1336,13 @@
       <c r="E27" s="10" t="n"/>
       <c r="F27" s="10" t="n"/>
       <c r="G27" s="11" t="n">
-        <v>7.999015182346275</v>
+        <v>6.889170497635929</v>
       </c>
       <c r="H27" s="11" t="n">
-        <v>27.22361730932283</v>
+        <v>36.36563417808039</v>
       </c>
       <c r="I27" s="11" t="n">
-        <v>32.07547882517483</v>
+        <v>29.18608564705882</v>
       </c>
       <c r="J27" s="10" t="n"/>
     </row>
@@ -1360,13 +1358,13 @@
       <c r="E28" s="10" t="n"/>
       <c r="F28" s="10" t="n"/>
       <c r="G28" s="11" t="n">
-        <v>4.682050540522233</v>
+        <v>4.715197797430405</v>
       </c>
       <c r="H28" s="11" t="n">
-        <v>16.78282109852865</v>
+        <v>17.83185481515893</v>
       </c>
       <c r="I28" s="11" t="n">
-        <v>16.85520402015944</v>
+        <v>17.47443304389261</v>
       </c>
       <c r="J28" s="10" t="n"/>
     </row>
@@ -1382,13 +1380,13 @@
       <c r="E29" s="10" t="n"/>
       <c r="F29" s="10" t="n"/>
       <c r="G29" s="11" t="n">
-        <v>3.133654760726173</v>
+        <v>3.196240666874038</v>
       </c>
       <c r="H29" s="11" t="n">
-        <v>9.979718148677026</v>
+        <v>10.18526991348173</v>
       </c>
       <c r="I29" s="11" t="n">
-        <v>9.686544422249289</v>
+        <v>9.885252807145758</v>
       </c>
       <c r="J29" s="10" t="n"/>
     </row>
@@ -1430,7 +1428,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Calendarized to CY2025 · Market data as of 2026-10-18 · $ in millions except per-share · NM = not meaningful, n/a = missing input</t>
+          <t>Calendarized to CY2025 · Market data as of 2026-11-01 · $ in millions except per-share · NM = not meaningful, n/a = missing input</t>
         </is>
       </c>
     </row>
@@ -2612,13 +2610,13 @@
         <v>3</v>
       </c>
       <c r="C5" s="7" t="n">
-        <v>8.883454913853628</v>
+        <v>7.856065682181051</v>
       </c>
       <c r="D5" s="7" t="n">
-        <v>48.62210211108567</v>
+        <v>42.08175284259329</v>
       </c>
       <c r="E5" s="7" t="n">
-        <v>32.07547882517483</v>
+        <v>23.84305946853147</v>
       </c>
       <c r="F5" s="12" t="n">
         <v>0.2088492352512746</v>
@@ -2655,11 +2653,11 @@
         <v>6</v>
       </c>
       <c r="C6" s="7" t="n">
-        <v>17.43608976547953</v>
+        <v>18.24668142334648</v>
       </c>
       <c r="D6" s="8" t="inlineStr"/>
       <c r="E6" s="7" t="n">
-        <v>58.03623578598857</v>
+        <v>60.68213667682251</v>
       </c>
       <c r="F6" s="12" t="n">
         <v>0.2341908156497334</v>
@@ -2696,13 +2694,13 @@
         <v>5</v>
       </c>
       <c r="C7" s="7" t="n">
-        <v>5.129153217228216</v>
+        <v>5.184206022372479</v>
       </c>
       <c r="D7" s="7" t="n">
-        <v>19.15528911864219</v>
+        <v>19.36088882578069</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>22.90427912566235</v>
+        <v>23.14480614730536</v>
       </c>
       <c r="F7" s="12" t="n">
         <v>0.09566540157649711</v>
@@ -2739,13 +2737,13 @@
         <v>4</v>
       </c>
       <c r="C8" s="7" t="n">
-        <v>4.113067471013871</v>
+        <v>4.372118641190823</v>
       </c>
       <c r="D8" s="7" t="n">
-        <v>32.90165920502642</v>
+        <v>53.01263921412894</v>
       </c>
       <c r="E8" s="7" t="n">
-        <v>17.15824815160536</v>
+        <v>17.48428569736987</v>
       </c>
       <c r="F8" s="12" t="n">
         <v>0.1089543920177844</v>
@@ -2859,7 +2857,7 @@
         </is>
       </c>
       <c r="B5" s="6" t="n">
-        <v>95431.83564799999</v>
+        <v>97389.510656</v>
       </c>
       <c r="C5" s="6" t="n">
         <v>6210</v>
@@ -2871,7 +2869,7 @@
         <v>1164</v>
       </c>
       <c r="F5" s="6" t="n">
-        <v>95046.83564799999</v>
+        <v>97004.510656</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -2891,7 +2889,7 @@
         </is>
       </c>
       <c r="B6" s="6" t="n">
-        <v>198096.093184</v>
+        <v>188606.906368</v>
       </c>
       <c r="C6" s="6" t="n">
         <v>14439</v>
@@ -2903,7 +2901,7 @@
         <v>2238</v>
       </c>
       <c r="F6" s="6" t="n">
-        <v>202970.093184</v>
+        <v>193480.906368</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -2923,7 +2921,7 @@
         </is>
       </c>
       <c r="B7" s="6" t="n">
-        <v>232832.548864</v>
+        <v>256424.001536</v>
       </c>
       <c r="C7" s="6" t="n">
         <v>745.471</v>
@@ -2935,7 +2933,7 @@
         <v>0</v>
       </c>
       <c r="F7" s="6" t="n">
-        <v>228347.894864</v>
+        <v>251939.347536</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -2955,7 +2953,7 @@
         </is>
       </c>
       <c r="B8" s="6" t="n">
-        <v>88731.025408</v>
+        <v>84479.58220800001</v>
       </c>
       <c r="C8" s="6" t="n">
         <v>983.449</v>
@@ -2967,7 +2965,7 @@
         <v>4073.531</v>
       </c>
       <c r="F8" s="6" t="n">
-        <v>85239.638408</v>
+        <v>80988.195208</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -2987,7 +2985,7 @@
         </is>
       </c>
       <c r="B9" s="6" t="n">
-        <v>13952.268288</v>
+        <v>15357.773824</v>
       </c>
       <c r="C9" s="6" t="n">
         <v>0</v>
@@ -2999,7 +2997,7 @@
         <v>0</v>
       </c>
       <c r="F9" s="6" t="n">
-        <v>13349.826288</v>
+        <v>14755.331824</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -3019,7 +3017,7 @@
         </is>
       </c>
       <c r="B10" s="6" t="n">
-        <v>11516.100608</v>
+        <v>11712.073728</v>
       </c>
       <c r="C10" s="6" t="n">
         <v>0</v>
@@ -3031,7 +3029,7 @@
         <v>821.552</v>
       </c>
       <c r="F10" s="6" t="n">
-        <v>9812.306608000001</v>
+        <v>10008.279728</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
@@ -3051,7 +3049,7 @@
         </is>
       </c>
       <c r="B11" s="6" t="n">
-        <v>27193.40544</v>
+        <v>28433.166336</v>
       </c>
       <c r="C11" s="6" t="n">
         <v>0</v>
@@ -3063,7 +3061,7 @@
         <v>1303.701</v>
       </c>
       <c r="F11" s="6" t="n">
-        <v>24806.16444</v>
+        <v>26045.925336</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
@@ -3083,7 +3081,7 @@
         </is>
       </c>
       <c r="B12" s="6" t="n">
-        <v>146777.391104</v>
+        <v>109105.840128</v>
       </c>
       <c r="C12" s="6" t="n">
         <v>1491</v>
@@ -3095,7 +3093,7 @@
         <v>2558</v>
       </c>
       <c r="F12" s="6" t="n">
-        <v>141984.391104</v>
+        <v>104312.840128</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
@@ -3115,7 +3113,7 @@
         </is>
       </c>
       <c r="B13" s="6" t="n">
-        <v>32736.966656</v>
+        <v>36404.711424</v>
       </c>
       <c r="C13" s="6" t="n">
         <v>350</v>
@@ -3127,7 +3125,7 @@
         <v>0</v>
       </c>
       <c r="F13" s="6" t="n">
-        <v>32228.966656</v>
+        <v>35896.711424</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
@@ -3147,7 +3145,7 @@
         </is>
       </c>
       <c r="B14" s="6" t="n">
-        <v>11341.821952</v>
+        <v>11907.922944</v>
       </c>
       <c r="C14" s="6" t="n">
         <v>0</v>
@@ -3159,7 +3157,7 @@
         <v>0</v>
       </c>
       <c r="F14" s="6" t="n">
-        <v>10971.821952</v>
+        <v>11537.922944</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
@@ -3179,7 +3177,7 @@
         </is>
       </c>
       <c r="B15" s="6" t="n">
-        <v>8824.434687999999</v>
+        <v>8917.103616</v>
       </c>
       <c r="C15" s="6" t="n">
         <v>81.25</v>
@@ -3191,7 +3189,7 @@
         <v>0</v>
       </c>
       <c r="F15" s="6" t="n">
-        <v>8633.767688</v>
+        <v>8726.436616000001</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
@@ -3211,7 +3209,7 @@
         </is>
       </c>
       <c r="B16" s="6" t="n">
-        <v>108253.151232</v>
+        <v>107985.01888</v>
       </c>
       <c r="C16" s="6" t="n">
         <v>2279.827</v>
@@ -3223,7 +3221,7 @@
         <v>1201.523</v>
       </c>
       <c r="F16" s="6" t="n">
-        <v>106503.292232</v>
+        <v>106235.15988</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
@@ -3243,7 +3241,7 @@
         </is>
       </c>
       <c r="B17" s="6" t="n">
-        <v>52607.311872</v>
+        <v>48531.775488</v>
       </c>
       <c r="C17" s="6" t="n">
         <v>989.5599999999999</v>
@@ -3255,7 +3253,7 @@
         <v>0</v>
       </c>
       <c r="F17" s="6" t="n">
-        <v>52357.359872</v>
+        <v>48281.823488</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
@@ -3275,7 +3273,7 @@
         </is>
       </c>
       <c r="B18" s="6" t="n">
-        <v>37529.174016</v>
+        <v>31487.526912</v>
       </c>
       <c r="C18" s="6" t="n">
         <v>992.287</v>
@@ -3287,7 +3285,7 @@
         <v>1788.007</v>
       </c>
       <c r="F18" s="6" t="n">
-        <v>36051.119016</v>
+        <v>30009.471912</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
@@ -3307,7 +3305,7 @@
         </is>
       </c>
       <c r="B19" s="6" t="n">
-        <v>50250.027008</v>
+        <v>50670.993408</v>
       </c>
       <c r="C19" s="6" t="n">
         <v>0</v>
@@ -3319,7 +3317,7 @@
         <v>5139.581</v>
       </c>
       <c r="F19" s="6" t="n">
-        <v>43689.213008</v>
+        <v>44110.179408</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
@@ -3339,7 +3337,7 @@
         </is>
       </c>
       <c r="B20" s="6" t="n">
-        <v>45985.210368</v>
+        <v>47674.621952</v>
       </c>
       <c r="C20" s="6" t="n">
         <v>2987</v>
@@ -3351,7 +3349,7 @@
         <v>3942</v>
       </c>
       <c r="F20" s="6" t="n">
-        <v>43529.210368</v>
+        <v>45218.621952</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
@@ -3371,7 +3369,7 @@
         </is>
       </c>
       <c r="B21" s="6" t="n">
-        <v>27483.109376</v>
+        <v>27865.344</v>
       </c>
       <c r="C21" s="6" t="n">
         <v>0</v>
@@ -3383,7 +3381,7 @@
         <v>6544.031</v>
       </c>
       <c r="F21" s="6" t="n">
-        <v>19666.201376</v>
+        <v>20048.436</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
@@ -3403,7 +3401,7 @@
         </is>
       </c>
       <c r="B22" s="6" t="n">
-        <v>33814.284288</v>
+        <v>38779.301888</v>
       </c>
       <c r="C22" s="6" t="n">
         <v>1696.355</v>
@@ -3415,7 +3413,7 @@
         <v>0</v>
       </c>
       <c r="F22" s="6" t="n">
-        <v>34582.285288</v>
+        <v>39547.302888</v>
       </c>
       <c r="G22" t="inlineStr">
         <is>

</xml_diff>